<commit_message>
talla el gestor de coordinación en la hoja de v2
Entran 18 requisitos y 112 días hábiles: nueve que ya estaban en la hoja
sin tallar y nueve nuevos que la banda del diagrama exige. El MVP pasa
de 76 requisitos y 525 días a 94 y 637.

Tres quedan en alerta y sin tallar, con la duda escrita: RF-105 porque
pide levantamiento y no construcción, RT-025 porque no acota el alcance
de la integración con prestadores, y RT-027 porque no es un requisito
sino la observación de que este gestor es el menos profundizado.

RF-075 y RT-023 se quedan fuera: son nivel 2 y 3. La columna K «Entra
en» marca la versión de cada requisito y queda dentro del autofiltro,
para separar el delta de v2 sin cambiar el significado de los colores.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/v2/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/v2/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Variables de monitoreo" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estimación por Requisitos'!$A$4:$Q$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estimación por Requisitos'!$A$4:$Q$196</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Requisitos Funcionales'!$A$1:$G$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Requisitos Técnicos'!$A$1:$F$53</definedName>
   </definedNames>
@@ -617,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -919,6 +919,15 @@
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1179,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q187"/>
+  <dimension ref="A1:Q196"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="14.45"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1190,6 +1199,7 @@
     <col width="12" customWidth="1" min="6" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="15"/>
@@ -1269,6 +1279,11 @@
           <t>Capacidad agéntica</t>
         </is>
       </c>
+      <c r="K4" s="51" t="inlineStr">
+        <is>
+          <t>Entra en</t>
+        </is>
+      </c>
       <c r="L4" s="52" t="inlineStr">
         <is>
           <t>Talla</t>
@@ -1329,6 +1344,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L5" s="56" t="inlineStr">
         <is>
           <t>S</t>
@@ -1386,6 +1406,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L6" s="56" t="inlineStr">
         <is>
           <t>M</t>
@@ -1445,6 +1470,11 @@
       <c r="J7" s="53" t="inlineStr">
         <is>
           <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="L7" s="56" t="inlineStr">
@@ -1507,6 +1537,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L8" s="56" t="inlineStr">
         <is>
           <t>XL</t>
@@ -1561,6 +1596,11 @@
         </is>
       </c>
       <c r="J9" s="53" t="n"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L9" s="91" t="inlineStr">
         <is>
           <t>🟨 Escala de referencia (no oficial para todas las tallas): M ≈ 5 días (medio sprint) y L ≈ 10 días (1 sprint) están tomados literalmente del Acta de Estimación de Costo y Releases (21-ago-2026). S (≈3 días) y XL (≈20 días, el doble de L, por la regla de coherencia de tallaje de Víctor Martínez) son un supuesto para completar la escala — ajústelos si el equipo define otro valor. 1 sprint = 10 días hábiles (estándar SuraHis).</t>
@@ -1648,6 +1688,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="57" t="inlineStr">
@@ -1693,6 +1738,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="53" t="inlineStr">
@@ -1738,6 +1788,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L13" s="90" t="inlineStr">
         <is>
           <t>Referencia de Épicas (usada por la columna "¿En MVP?")</t>
@@ -1788,6 +1843,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L14" s="52" t="inlineStr">
         <is>
           <t>Épica / Gestor-Frente</t>
@@ -1867,17 +1927,22 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L15" s="58" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
       <c r="M15" s="58">
-        <f>COUNTIFS($C$5:$C$187,L15,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L15,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N15" s="58">
-        <f>COUNTIFS($C$5:$C$187,L15,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L15,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O15" s="58" t="inlineStr">
@@ -1940,17 +2005,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L16" s="58" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
       <c r="M16" s="58">
-        <f>COUNTIFS($C$5:$C$187,L16,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L16,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N16" s="58">
-        <f>COUNTIFS($C$5:$C$187,L16,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L16,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O16" s="58" t="inlineStr">
@@ -2013,17 +2083,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L17" s="60" t="inlineStr">
         <is>
           <t>Gestor de Evaluación</t>
         </is>
       </c>
       <c r="M17" s="60">
-        <f>COUNTIFS($C$5:$C$187,L17,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L17,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N17" s="60">
-        <f>COUNTIFS($C$5:$C$187,L17,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L17,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O17" s="60" t="inlineStr">
@@ -2086,17 +2161,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L18" s="60" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
       <c r="M18" s="60">
-        <f>COUNTIFS($C$5:$C$187,L18,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L18,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N18" s="60">
-        <f>COUNTIFS($C$5:$C$187,L18,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L18,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O18" s="60" t="inlineStr">
@@ -2159,32 +2239,37 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L19" s="62" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
         </is>
       </c>
       <c r="M19" s="62">
-        <f>COUNTIFS($C$5:$C$187,L19,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L19,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N19" s="62">
-        <f>COUNTIFS($C$5:$C$187,L19,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L19,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O19" s="62" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="P19" s="62" t="inlineStr">
         <is>
-          <t>No aplica (absorbido por Core)</t>
+          <t>Release 3 (dentro del MVP)</t>
         </is>
       </c>
       <c r="Q19" s="57" t="inlineStr">
         <is>
-          <t>Decidido el 03-ago-2026 (con Viviana Monsalve): NO se implementa como gestor agéntico independiente. La asignación de prestador queda encapsulada en SuraHis (Core), principio KISS.</t>
+          <t>Se retoma en v2 como gestor propio, revirtiendo la decisión del 03-ago-2026 que lo dejaba encapsulado en SuraHis. Entra solo su nivel 1 determinístico: reglas duras, ranking de red y bandeja human in the loop. El asistente explicativo con modelo y el componente conversacional (RF-075, RT-023) quedan fuera.</t>
         </is>
       </c>
     </row>
@@ -2230,11 +2315,11 @@
         </is>
       </c>
       <c r="M20" s="60">
-        <f>COUNTIFS($C$5:$C$187,L20,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L20,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N20" s="60">
-        <f>COUNTIFS($C$5:$C$187,L20,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L20,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O20" s="60" t="inlineStr">
@@ -2295,11 +2380,11 @@
         </is>
       </c>
       <c r="M21" s="60">
-        <f>COUNTIFS($C$5:$C$187,L21,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L21,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N21" s="60">
-        <f>COUNTIFS($C$5:$C$187,L21,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L21,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O21" s="60" t="inlineStr">
@@ -2358,17 +2443,22 @@
         </is>
       </c>
       <c r="J22" s="53" t="n"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L22" s="58" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
       <c r="M22" s="58">
-        <f>COUNTIFS($C$5:$C$187,L22,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L22,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N22" s="58">
-        <f>COUNTIFS($C$5:$C$187,L22,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L22,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O22" s="58" t="inlineStr">
@@ -2429,11 +2519,11 @@
         </is>
       </c>
       <c r="M23" s="60">
-        <f>COUNTIFS($C$5:$C$187,L23,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L23,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N23" s="60">
-        <f>COUNTIFS($C$5:$C$187,L23,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L23,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O23" s="60" t="inlineStr">
@@ -2496,17 +2586,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L24" s="62" t="inlineStr">
         <is>
           <t>NEXO (Asesores)</t>
         </is>
       </c>
       <c r="M24" s="62">
-        <f>COUNTIFS($C$5:$C$187,L24,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L24,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N24" s="62">
-        <f>COUNTIFS($C$5:$C$187,L24,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L24,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O24" s="62" t="inlineStr">
@@ -2571,17 +2666,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L25" s="62" t="inlineStr">
         <is>
           <t>Gestor de Prestación</t>
         </is>
       </c>
       <c r="M25" s="62">
-        <f>COUNTIFS($C$5:$C$187,L25,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L25,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N25" s="62">
-        <f>COUNTIFS($C$5:$C$187,L25,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L25,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O25" s="62" t="inlineStr">
@@ -2648,17 +2748,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L26" s="62" t="inlineStr">
         <is>
           <t>AVA (Asesores — AVA)</t>
         </is>
       </c>
       <c r="M26" s="62">
-        <f>COUNTIFS($C$5:$C$187,L26,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L26,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N26" s="62">
-        <f>COUNTIFS($C$5:$C$187,L26,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L26,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O26" s="62" t="inlineStr">
@@ -2721,17 +2826,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L27" s="60" t="inlineStr">
         <is>
           <t>Transversal</t>
         </is>
       </c>
       <c r="M27" s="60">
-        <f>COUNTIFS($C$5:$C$187,L27,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L27,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N27" s="60">
-        <f>COUNTIFS($C$5:$C$187,L27,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L27,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O27" s="60" t="inlineStr">
@@ -2794,17 +2904,22 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L28" s="62" t="inlineStr">
         <is>
           <t>Gestor de Finalización</t>
         </is>
       </c>
       <c r="M28" s="62">
-        <f>COUNTIFS($C$5:$C$187,L28,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L28,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N28" s="62">
-        <f>COUNTIFS($C$5:$C$187,L28,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L28,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O28" s="62" t="inlineStr">
@@ -2867,17 +2982,22 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L29" s="62" t="inlineStr">
         <is>
           <t>Surahis</t>
         </is>
       </c>
       <c r="M29" s="62">
-        <f>COUNTIFS($C$5:$C$187,L29,$B$5:$B$187,"Funcional")</f>
+        <f>COUNTIFS($C$5:$C$196,L29,$B$5:$B$196,"Funcional")</f>
         <v/>
       </c>
       <c r="N29" s="62">
-        <f>COUNTIFS($C$5:$C$187,L29,$B$5:$B$187,"Técnico")</f>
+        <f>COUNTIFS($C$5:$C$196,L29,$B$5:$B$196,"Técnico")</f>
         <v/>
       </c>
       <c r="O29" s="62" t="inlineStr">
@@ -2940,6 +3060,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="53" t="inlineStr">
@@ -2983,6 +3108,11 @@
       <c r="J31" s="53" t="inlineStr">
         <is>
           <t>Agéntica</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="L31" s="115" t="n"/>
@@ -3036,6 +3166,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L32" s="108" t="inlineStr">
         <is>
           <t>Leyenda y criterio de esta estimación (Tech and Solve)</t>
@@ -3091,6 +3226,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L33" s="116" t="inlineStr">
         <is>
           <t>Fila adicionada</t>
@@ -3098,7 +3238,7 @@
       </c>
       <c r="M33" s="110" t="inlineStr">
         <is>
-          <t>Requisito funcional nuevo, RF-109 a RF-129. Elementos que el dibujo del MVP y la vista de tecnología exigen y que la hoja no tenía.</t>
+          <t>Requisito funcional o técnico nuevo. En v1, RF-109 a RF-129, por el dibujo del MVP y la vista de tecnología. En v2, RF-135 a RF-139 y RT-055 a RT-058, por lo que la banda del Gestor de Coordinación exige y la hoja no tenía.</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3285,7 @@
       </c>
       <c r="M34" s="110" t="inlineStr">
         <is>
-          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones. Son 11.</t>
+          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones. Son 14: 11 de v1 y 3 que aparecen al abrir Coordinación.</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3332,7 @@
       </c>
       <c r="M35" s="110" t="inlineStr">
         <is>
-          <t>Requisito que entra al MVP con una salvedad sobre qué cubre la talla, o cuya duda ya se cerró con una decisión del equipo; en ambos casos queda escrita en Observaciones. Son 9.</t>
+          <t>Requisito que entra al MVP con una salvedad sobre qué cubre la talla, o cuya duda ya se cerró con una decisión del equipo; en ambos casos queda escrita en Observaciones. Son 11.</t>
         </is>
       </c>
     </row>
@@ -3326,8 +3466,16 @@
       </c>
       <c r="I38" s="53" t="n"/>
       <c r="J38" s="53" t="n"/>
-      <c r="L38" s="115" t="n"/>
-      <c r="M38" s="115" t="n"/>
+      <c r="L38" s="120" t="inlineStr">
+        <is>
+          <t>Columna «Entra en»</t>
+        </is>
+      </c>
+      <c r="M38" s="110" t="inlineStr">
+        <is>
+          <t>Filtro rápido de versión. «v1» son los requisitos que ya estaban dentro del alcance estimado; «v2» son los 18 del Gestor de Coordinación que entran ahora más los 3 que quedaron en alerta. Las filas fuera del MVP quedan en blanco. El color de fila conserva el significado que tenía en v1.</t>
+        </is>
+      </c>
       <c r="N38" s="115" t="n"/>
       <c r="O38" s="115" t="n"/>
       <c r="P38" s="115" t="n"/>
@@ -3423,7 +3571,7 @@
       </c>
       <c r="M40" s="110" t="inlineStr">
         <is>
-          <t>76 requisitos del MVP tallados: 525 días hábiles, 52 sprints de un frente, con la escala de la propia hoja. La suma va sin margen de incertidumbre. Reparto: Gestor de Evaluación 138 d · Gestor de Monitoreo 97 d · Gestor de Solicitud 84 d · Transversal (principios) 59 d · Siniestro Integral 52 d · Transversal 50 d · Canales / Front Externos 43 d · Interoperabilidad (Prestadores) 2 d.</t>
+          <t>94 requisitos del MVP tallados: 637 días hábiles, 64 sprints de un frente, con la escala de la propia hoja. La suma va sin margen de incertidumbre. Reparto: Gestor de Evaluación 138 d · Gestor de Coordinación 112 d · Gestor de Monitoreo (Torre de Control) 97 d · Gestor de Solicitud 84 d · Transversal / Principios generales 59 d · Siniestro Integral 52 d · Transversal 50 d · Canales / Front Externos 43 d · Interoperabilidad (Prestadores) 2 d.</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3639,11 @@
           <t xml:space="preserve">Si el asegurado sugiere un prestador y está en convenio para los servicios que se requieren se genera la autorización sin problema a ese prestador </t>
         </is>
       </c>
-      <c r="E42" s="54" t="n"/>
+      <c r="E42" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F42" s="53">
         <f>IF($E42="",0,INDEX($M$5:$M$8,MATCH($E42,$L$5:$L$8,0)))</f>
         <v/>
@@ -3505,7 +3657,16 @@
         <v/>
       </c>
       <c r="I42" s="53" t="n"/>
-      <c r="J42" s="53" t="n"/>
+      <c r="J42" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
       <c r="L42" s="108" t="inlineStr">
         <is>
           <t>Criterio de alcance</t>
@@ -3544,7 +3705,11 @@
 2. Cuando el asegurado solicita una autorización y en el ordenamiento esta un proveedor que atiende diferente al sugerido por el asegurado, se debe dar prioridad al que sugiere el asegurado</t>
         </is>
       </c>
-      <c r="E43" s="54" t="n"/>
+      <c r="E43" s="54" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="F43" s="53">
         <f>IF($E43="",0,INDEX($M$5:$M$8,MATCH($E43,$L$5:$L$8,0)))</f>
         <v/>
@@ -3558,7 +3723,16 @@
         <v/>
       </c>
       <c r="I43" s="53" t="n"/>
-      <c r="J43" s="53" t="n"/>
+      <c r="J43" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
       <c r="L43" s="120" t="inlineStr">
         <is>
           <t>Qué entra</t>
@@ -3566,46 +3740,63 @@
       </c>
       <c r="M43" s="110" t="inlineStr">
         <is>
-          <t>La pertenencia al MVP se decidió requisito por requisito contra «resumen-arquitectura-gestores — Arquitectura MVP» y «arquitectura-tecnologia», no contra la columna «¿En MVP?», que se deriva por épica y por eso marca «Sí» a épicas donde solo una parte entra. Entran Solicitud, Evaluación, Siniestro Integral, los canales que el MVP habilita, las capas 1 y 2 de la torre, el acceso al dato vía el core y los transversales del ciclo de mejora y del plano de control. Quedan fuera Coordinación, Prestación, Finalización, Asignación, Nexo, AVA, la interoperabilidad de autorizaciones y las capas 3, 4 y 5 de la torre.</t>
+          <t>La pertenencia al MVP se decidió requisito por requisito contra «resumen-arquitectura-gestores — Arquitectura MVP» y «arquitectura-tecnologia», no contra la columna «¿En MVP?», que se deriva por épica y por eso marca «Sí» a épicas donde solo una parte entra. Entran Solicitud, Evaluación, Coordinación en su nivel 1 determinístico, Siniestro Integral, los canales que el MVP habilita, las capas 1 y 2 de la torre, el acceso al dato vía el core y los transversales del ciclo de mejora y del plano de control. Quedan fuera Prestación, Finalización, Asignación, Nexo, AVA, la interoperabilidad de autorizaciones, las capas 3, 4 y 5 de la torre, y los niveles 2 y 3 de Coordinación.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="57" t="inlineStr">
+      <c r="A44" s="105" t="inlineStr">
         <is>
           <t>RF-040</t>
         </is>
       </c>
-      <c r="B44" s="57" t="inlineStr">
+      <c r="B44" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C44" s="57" t="inlineStr">
+      <c r="C44" s="105" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
         </is>
       </c>
-      <c r="D44" s="57" t="inlineStr">
+      <c r="D44" s="105" t="inlineStr">
         <is>
           <t>Criterios de priorización de prestadores: quejas (Medallia), satisfacción, disponibilidad de citas, "suficiencia de la red" y tarifa del prestador.</t>
         </is>
       </c>
-      <c r="E44" s="54" t="n"/>
-      <c r="F44" s="53">
+      <c r="E44" s="123" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F44" s="105">
         <f>IF($E44="",0,INDEX($M$5:$M$8,MATCH($E44,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G44" s="53">
+      <c r="G44" s="105">
         <f>IF($F44=0,0,$F44/10)</f>
         <v/>
       </c>
-      <c r="H44" s="53">
+      <c r="H44" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C44,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I44" s="53" t="n"/>
-      <c r="J44" s="53" t="n"/>
+      <c r="I44" s="105" t="inlineStr">
+        <is>
+          <t>La talla cubre el motor de ordenamiento y el consumo de los criterios que hoy son consultables. Las cinco fuentes —Medallia, satisfacción, agenda de citas, suficiencia de red y tarifa— tienen dueños distintos; habilitar las que no estén expuestas no está en esta talla y su plazo lo declara su dueño.</t>
+        </is>
+      </c>
+      <c r="J44" s="105" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K44" s="124" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
       <c r="L44" s="115" t="n"/>
       <c r="M44" s="115" t="n"/>
       <c r="N44" s="115" t="n"/>
@@ -3634,7 +3825,11 @@
           <t>Si el prestador elegido no tiene convenio vigente, se asigna automáticamente el mejor rankeado y se notifica al cliente.</t>
         </is>
       </c>
-      <c r="E45" s="54" t="n"/>
+      <c r="E45" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F45" s="53">
         <f>IF($E45="",0,INDEX($M$5:$M$8,MATCH($E45,$L$5:$L$8,0)))</f>
         <v/>
@@ -3648,7 +3843,16 @@
         <v/>
       </c>
       <c r="I45" s="53" t="n"/>
-      <c r="J45" s="53" t="n"/>
+      <c r="J45" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
       <c r="L45" s="108" t="inlineStr">
         <is>
           <t>Tres cosas que conviene saber antes de leer el total</t>
@@ -3681,7 +3885,11 @@
           <t>Si no hay red contratada en la ciudad, se escala a Convenios (bandeja de convenios en SuraHis).</t>
         </is>
       </c>
-      <c r="E46" s="54" t="n"/>
+      <c r="E46" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F46" s="53">
         <f>IF($E46="",0,INDEX($M$5:$M$8,MATCH($E46,$L$5:$L$8,0)))</f>
         <v/>
@@ -3695,7 +3903,16 @@
         <v/>
       </c>
       <c r="I46" s="53" t="n"/>
-      <c r="J46" s="53" t="n"/>
+      <c r="J46" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
       <c r="L46" s="120" t="inlineStr">
         <is>
           <t>La escala se contradice</t>
@@ -3703,7 +3920,7 @@
       </c>
       <c r="M46" s="110" t="inlineStr">
         <is>
-          <t>La tabla de tallaje dice S = 2 días y la nota de al lado dice S ≈ 3 días. Se usó la tabla, porque es la que alimenta la fórmula de la columna F. Si el equipo confirma los 3 días, el total sube 15 días (hay 15 requisitos en S).</t>
+          <t>La tabla de tallaje dice S = 2 días y la nota de al lado dice S ≈ 3 días. Se usó la tabla, porque es la que alimenta la fórmula de la columna F. Si el equipo confirma los 3 días, el total sube 21 días (hay 21 requisitos en S).</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3945,11 @@
           <t>mapear automáticamente la autorización contra el convenio/tarifa para pagar más rápido y reducir glosas.</t>
         </is>
       </c>
-      <c r="E47" s="54" t="n"/>
+      <c r="E47" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F47" s="53">
         <f>IF($E47="",0,INDEX($M$5:$M$8,MATCH($E47,$L$5:$L$8,0)))</f>
         <v/>
@@ -3742,7 +3963,16 @@
         <v/>
       </c>
       <c r="I47" s="53" t="n"/>
-      <c r="J47" s="53" t="n"/>
+      <c r="J47" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
       <c r="L47" s="120" t="inlineStr">
         <is>
           <t>Funcionales y técnicos se suman</t>
@@ -3750,7 +3980,7 @@
       </c>
       <c r="M47" s="110" t="inlineStr">
         <is>
-          <t>La hoja talla por separado el requisito funcional y el técnico, y así se respetó. Hay pares que describen la misma capacidad —RF-021 con RT-018, RF-024 con RT-020, RF-025 con RT-021, RF-001 con RT-011, RF-011 con RT-017—. Si el equipo decide contarlos una sola vez, el total baja hasta 32 días.</t>
+          <t>La hoja talla por separado el requisito funcional y el técnico, y así se respetó. Hay pares que describen la misma capacidad —RF-021 con RT-018, RF-024 con RT-020, RF-025 con RT-021, RF-001 con RT-011, RF-011 con RT-017, y en Coordinación RF-039 con RT-022 y RF-040 con RT-056—. Si el equipo decide contarlos una sola vez, el total baja hasta 47 días.</t>
         </is>
       </c>
     </row>
@@ -3998,17 +4228,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L52" s="114" t="inlineStr">
         <is>
           <t>Agéntica</t>
         </is>
       </c>
       <c r="M52" s="121">
-        <f>COUNTIF($J$5:$J$187,$L52)</f>
+        <f>COUNTIF($J$5:$J$196,$L52)</f>
         <v/>
       </c>
       <c r="N52" s="121">
-        <f>SUMIF($J$5:$J$187,$L52,$F$5:$F$187)</f>
+        <f>SUMIF($J$5:$J$196,$L52,$F$5:$F$196)</f>
         <v/>
       </c>
       <c r="O52" s="121">
@@ -4063,11 +4298,11 @@
         </is>
       </c>
       <c r="M53" s="121">
-        <f>COUNTIF($J$5:$J$187,$L53)</f>
+        <f>COUNTIF($J$5:$J$196,$L53)</f>
         <v/>
       </c>
       <c r="N53" s="121">
-        <f>SUMIF($J$5:$J$187,$L53,$F$5:$F$187)</f>
+        <f>SUMIF($J$5:$J$196,$L53,$F$5:$F$196)</f>
         <v/>
       </c>
       <c r="O53" s="121">
@@ -4124,17 +4359,22 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
       <c r="L54" s="114" t="inlineStr">
         <is>
           <t>Determinística</t>
         </is>
       </c>
       <c r="M54" s="121">
-        <f>COUNTIF($J$5:$J$187,$L54)</f>
+        <f>COUNTIF($J$5:$J$196,$L54)</f>
         <v/>
       </c>
       <c r="N54" s="121">
-        <f>SUMIF($J$5:$J$187,$L54,$F$5:$F$187)</f>
+        <f>SUMIF($J$5:$J$196,$L54,$F$5:$F$196)</f>
         <v/>
       </c>
       <c r="O54" s="121">
@@ -4341,6 +4581,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="53" t="inlineStr">
@@ -4460,6 +4705,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="105" t="inlineStr">
@@ -4507,6 +4757,11 @@
       <c r="J62" s="53" t="inlineStr">
         <is>
           <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -4965,6 +5220,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="53" t="inlineStr">
@@ -5228,6 +5488,11 @@
         </is>
       </c>
       <c r="J81" s="53" t="n"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="57" t="inlineStr">
@@ -5569,6 +5834,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="53" t="inlineStr">
@@ -5988,6 +6258,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="30" customHeight="1">
       <c r="A102" s="57" t="inlineStr">
@@ -6249,41 +6524,50 @@
       <c r="J108" s="53" t="n"/>
     </row>
     <row r="109" ht="30" customHeight="1">
-      <c r="A109" s="53" t="inlineStr">
+      <c r="A109" s="106" t="inlineStr">
         <is>
           <t>RF-105</t>
         </is>
       </c>
-      <c r="B109" s="53" t="inlineStr">
+      <c r="B109" s="106" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C109" s="53" t="inlineStr">
+      <c r="C109" s="106" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
         </is>
       </c>
-      <c r="D109" s="53" t="inlineStr">
+      <c r="D109" s="106" t="inlineStr">
         <is>
           <t>Registrar los requisitos funcionales de cara a la asignación de proveedor, cambio de proveedor y lo que la IA podrá interactuar con el cliente</t>
         </is>
       </c>
-      <c r="E109" s="54" t="n"/>
-      <c r="F109" s="53">
+      <c r="E109" s="107" t="n"/>
+      <c r="F109" s="106">
         <f>IF($E109="",0,INDEX($M$5:$M$8,MATCH($E109,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G109" s="53">
+      <c r="G109" s="106">
         <f>IF($F109=0,0,$F109/10)</f>
         <v/>
       </c>
-      <c r="H109" s="53">
+      <c r="H109" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C109,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I109" s="53" t="n"/>
-      <c r="J109" s="53" t="n"/>
+      <c r="I109" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No estimable como está redactado. Pide «registrar los requisitos funcionales» de la asignación y del cambio de proveedor, es decir es un requisito sobre el levantamiento y no sobre la construcción. La parte que sí es construible quedó tallada en RF-038, RF-039 y RF-139; la interacción de la IA con el cliente pertenece al nivel 2, fuera de este alcance.</t>
+        </is>
+      </c>
+      <c r="J109" s="106" t="n"/>
+      <c r="K109" s="125" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="30" customHeight="1">
       <c r="A110" s="57" t="inlineStr">
@@ -6440,6 +6724,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="30" customHeight="1">
       <c r="A114" s="57" t="inlineStr">
@@ -6483,6 +6772,11 @@
       <c r="J114" s="53" t="inlineStr">
         <is>
           <t>Habilitadora</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -6526,6 +6820,11 @@
         </is>
       </c>
       <c r="J115" s="53" t="n"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="30" customHeight="1">
       <c r="A116" s="57" t="inlineStr">
@@ -6571,6 +6870,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="30" customHeight="1">
       <c r="A117" s="53" t="inlineStr">
@@ -6616,6 +6920,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="30" customHeight="1">
       <c r="A118" s="57" t="inlineStr">
@@ -6661,6 +6970,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="30" customHeight="1">
       <c r="A119" s="53" t="inlineStr">
@@ -6706,6 +7020,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="30" customHeight="1">
       <c r="A120" s="105" t="inlineStr">
@@ -6755,6 +7074,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="53" t="inlineStr">
@@ -6800,6 +7124,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="30" customHeight="1">
       <c r="A122" s="57" t="inlineStr">
@@ -6845,6 +7174,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="30" customHeight="1">
       <c r="A123" s="53" t="inlineStr">
@@ -6888,6 +7222,11 @@
       <c r="J123" s="53" t="inlineStr">
         <is>
           <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -6931,6 +7270,11 @@
         </is>
       </c>
       <c r="J124" s="53" t="n"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="30" customHeight="1">
       <c r="A125" s="53" t="inlineStr">
@@ -6974,6 +7318,11 @@
       <c r="J125" s="53" t="inlineStr">
         <is>
           <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -7058,6 +7407,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="30" customHeight="1">
       <c r="A128" s="106" t="inlineStr">
@@ -7099,6 +7453,11 @@
         </is>
       </c>
       <c r="J128" s="53" t="n"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="30" customHeight="1">
       <c r="A129" s="53" t="inlineStr">
@@ -7144,6 +7503,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="30" customHeight="1">
       <c r="A130" s="57" t="inlineStr">
@@ -7187,6 +7551,11 @@
       <c r="J130" s="53" t="inlineStr">
         <is>
           <t>Agéntica</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -7230,6 +7599,11 @@
         </is>
       </c>
       <c r="J131" s="53" t="n"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="30" customHeight="1">
       <c r="A132" s="57" t="inlineStr">
@@ -7275,6 +7649,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="30" customHeight="1">
       <c r="A133" s="53" t="inlineStr">
@@ -7320,6 +7699,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="30" customHeight="1">
       <c r="A134" s="57" t="inlineStr">
@@ -7342,7 +7726,11 @@
           <t>Arranca con motor 100% determinístico (reglas duras de elegibilidad, convenios, capacidad, ubicación y costo).</t>
         </is>
       </c>
-      <c r="E134" s="54" t="n"/>
+      <c r="E134" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F134" s="53">
         <f>IF($E134="",0,INDEX($M$5:$M$8,MATCH($E134,$L$5:$L$8,0)))</f>
         <v/>
@@ -7356,7 +7744,16 @@
         <v/>
       </c>
       <c r="I134" s="53" t="n"/>
-      <c r="J134" s="53" t="n"/>
+      <c r="J134" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="30" customHeight="1">
       <c r="A135" s="53" t="inlineStr">
@@ -7396,78 +7793,104 @@
       <c r="J135" s="53" t="n"/>
     </row>
     <row r="136" ht="30" customHeight="1">
-      <c r="A136" s="57" t="inlineStr">
+      <c r="A136" s="105" t="inlineStr">
         <is>
           <t>RT-024</t>
         </is>
       </c>
-      <c r="B136" s="57" t="inlineStr">
+      <c r="B136" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C136" s="57" t="inlineStr">
+      <c r="C136" s="105" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
         </is>
       </c>
-      <c r="D136" s="57" t="inlineStr">
+      <c r="D136" s="105" t="inlineStr">
         <is>
           <t>Niveles de madurez agéntica: Nivel 1 determinístico → Nivel 2 + asistente explicativo → Nivel 3 agente autónomo (futuro, fuera de alcance actual).</t>
         </is>
       </c>
-      <c r="E136" s="54" t="n"/>
-      <c r="F136" s="53">
+      <c r="E136" s="123" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F136" s="105">
         <f>IF($E136="",0,INDEX($M$5:$M$8,MATCH($E136,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G136" s="53">
+      <c r="G136" s="105">
         <f>IF($F136=0,0,$F136/10)</f>
         <v/>
       </c>
-      <c r="H136" s="53">
+      <c r="H136" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C136,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I136" s="53" t="n"/>
-      <c r="J136" s="53" t="n"/>
+      <c r="I136" s="105" t="inlineStr">
+        <is>
+          <t>Entra solo como costura: el motor determinístico queda detrás de una interfaz para que el nivel 2 —asistente explicativo con modelo— no obligue a rehacerlo. El nivel 2 y el nivel 3 quedan fuera del MVP.</t>
+        </is>
+      </c>
+      <c r="J136" s="105" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
+      <c r="K136" s="124" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="30" customHeight="1">
-      <c r="A137" s="53" t="inlineStr">
+      <c r="A137" s="106" t="inlineStr">
         <is>
           <t>RT-025</t>
         </is>
       </c>
-      <c r="B137" s="53" t="inlineStr">
+      <c r="B137" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C137" s="53" t="inlineStr">
+      <c r="C137" s="106" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
         </is>
       </c>
-      <c r="D137" s="53" t="inlineStr">
+      <c r="D137" s="106" t="inlineStr">
         <is>
           <t>Integración con prestadores externos preferiblemente vía API con retroalimentación de estados.</t>
         </is>
       </c>
-      <c r="E137" s="54" t="n"/>
-      <c r="F137" s="53">
+      <c r="E137" s="107" t="n"/>
+      <c r="F137" s="106">
         <f>IF($E137="",0,INDEX($M$5:$M$8,MATCH($E137,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G137" s="53">
+      <c r="G137" s="106">
         <f>IF($F137=0,0,$F137/10)</f>
         <v/>
       </c>
-      <c r="H137" s="53">
+      <c r="H137" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C137,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I137" s="53" t="n"/>
-      <c r="J137" s="53" t="n"/>
+      <c r="I137" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No estimable: «preferiblemente vía API» no acota el alcance ni nombra los prestadores a integrar, y la retroalimentación de estados desde el prestador pertenece a la épica de Interoperabilidad, cuyo plazo declara su dueño.</t>
+        </is>
+      </c>
+      <c r="J137" s="106" t="n"/>
+      <c r="K137" s="125" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="30" customHeight="1">
       <c r="A138" s="57" t="inlineStr">
@@ -7490,7 +7913,11 @@
           <t>Bandeja "human in the loop" para casos donde ni las reglas ni la recomendación logran asignar un prestador.</t>
         </is>
       </c>
-      <c r="E138" s="54" t="n"/>
+      <c r="E138" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F138" s="53">
         <f>IF($E138="",0,INDEX($M$5:$M$8,MATCH($E138,$L$5:$L$8,0)))</f>
         <v/>
@@ -7504,44 +7931,62 @@
         <v/>
       </c>
       <c r="I138" s="53" t="n"/>
-      <c r="J138" s="53" t="n"/>
+      <c r="J138" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="30" customHeight="1">
-      <c r="A139" s="53" t="inlineStr">
+      <c r="A139" s="106" t="inlineStr">
         <is>
           <t>RT-027</t>
         </is>
       </c>
-      <c r="B139" s="53" t="inlineStr">
+      <c r="B139" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C139" s="53" t="inlineStr">
+      <c r="C139" s="106" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
         </is>
       </c>
-      <c r="D139" s="53" t="inlineStr">
+      <c r="D139" s="106" t="inlineStr">
         <is>
           <t>Es uno de los gestores menos profundizados técnicamente a la fecha — "no se ha hecho zoom" todavía.</t>
         </is>
       </c>
-      <c r="E139" s="54" t="n"/>
-      <c r="F139" s="53">
+      <c r="E139" s="107" t="n"/>
+      <c r="F139" s="106">
         <f>IF($E139="",0,INDEX($M$5:$M$8,MATCH($E139,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G139" s="53">
+      <c r="G139" s="106">
         <f>IF($F139=0,0,$F139/10)</f>
         <v/>
       </c>
-      <c r="H139" s="53">
+      <c r="H139" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C139,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I139" s="53" t="n"/>
-      <c r="J139" s="53" t="n"/>
+      <c r="I139" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No es un requisito sino la observación de que el gestor es el menos profundizado técnicamente. Es el riesgo principal de esta estimación y se declara como tal: la talla se construyó desde el dibujo y desde las reglas escritas, no desde un diseño detallado.</t>
+        </is>
+      </c>
+      <c r="J139" s="106" t="n"/>
+      <c r="K139" s="125" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="30" customHeight="1">
       <c r="A140" s="57" t="inlineStr">
@@ -7661,6 +8106,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="30" customHeight="1">
       <c r="A143" s="53" t="inlineStr">
@@ -7704,6 +8154,11 @@
       <c r="J143" s="53" t="inlineStr">
         <is>
           <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -7932,6 +8387,11 @@
         </is>
       </c>
       <c r="J149" s="53" t="n"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="30" customHeight="1">
       <c r="A150" s="106" t="inlineStr">
@@ -7973,6 +8433,11 @@
         </is>
       </c>
       <c r="J150" s="53" t="n"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="53" t="inlineStr">
@@ -8162,6 +8627,11 @@
         </is>
       </c>
       <c r="J155" s="53" t="n"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="30" customHeight="1">
       <c r="A156" s="57" t="inlineStr">
@@ -8207,6 +8677,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="105" t="inlineStr">
@@ -8254,6 +8729,11 @@
       <c r="J157" s="53" t="inlineStr">
         <is>
           <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
     </row>
@@ -8449,6 +8929,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="30" customHeight="1">
       <c r="A163" s="106" t="inlineStr">
@@ -8490,6 +8975,11 @@
         </is>
       </c>
       <c r="J163" s="53" t="n"/>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="30" customHeight="1">
       <c r="A164" s="57" t="inlineStr">
@@ -8535,6 +9025,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="30" customHeight="1">
       <c r="A165" s="53" t="inlineStr">
@@ -8580,6 +9075,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="57" t="inlineStr">
@@ -8625,6 +9125,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="30" customHeight="1">
       <c r="A167" s="98" t="inlineStr">
@@ -8670,6 +9175,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="30" customHeight="1">
       <c r="A168" s="98" t="inlineStr">
@@ -8715,6 +9225,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="30" customHeight="1">
       <c r="A169" s="98" t="inlineStr">
@@ -8760,6 +9275,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="30" customHeight="1">
       <c r="A170" s="98" t="inlineStr">
@@ -8805,6 +9325,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="98" t="inlineStr">
@@ -8850,6 +9375,11 @@
           <t>Agéntica</t>
         </is>
       </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="30" customHeight="1">
       <c r="A172" s="98" t="inlineStr">
@@ -8895,6 +9425,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="30" customHeight="1">
       <c r="A173" s="98" t="inlineStr">
@@ -8940,6 +9475,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="30" customHeight="1">
       <c r="A174" s="98" t="inlineStr">
@@ -8985,6 +9525,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="98" t="inlineStr">
@@ -9030,6 +9575,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="30" customHeight="1">
       <c r="A176" s="98" t="inlineStr">
@@ -9075,6 +9625,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="30" customHeight="1">
       <c r="A177" s="98" t="inlineStr">
@@ -9120,6 +9675,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="30" customHeight="1">
       <c r="A178" s="98" t="inlineStr">
@@ -9165,6 +9725,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="30" customHeight="1">
       <c r="A179" s="98" t="inlineStr">
@@ -9210,6 +9775,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="30" customHeight="1">
       <c r="A180" s="98" t="inlineStr">
@@ -9255,6 +9825,11 @@
           <t>Determinística</t>
         </is>
       </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="30" customHeight="1">
       <c r="A181" s="98" t="inlineStr">
@@ -9300,6 +9875,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="30" customHeight="1">
       <c r="A182" s="98" t="inlineStr">
@@ -9345,6 +9925,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="30" customHeight="1">
       <c r="A183" s="98" t="inlineStr">
@@ -9390,6 +9975,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="30" customHeight="1">
       <c r="A184" s="98" t="inlineStr">
@@ -9435,6 +10025,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="30" customHeight="1">
       <c r="A185" s="98" t="inlineStr">
@@ -9480,6 +10075,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="30" customHeight="1">
       <c r="A186" s="98" t="inlineStr">
@@ -9525,6 +10125,11 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="30" customHeight="1">
       <c r="A187" s="98" t="inlineStr">
@@ -9570,9 +10175,464 @@
           <t>Habilitadora</t>
         </is>
       </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="30" customHeight="1">
+      <c r="A188" s="98" t="inlineStr">
+        <is>
+          <t>RF-135</t>
+        </is>
+      </c>
+      <c r="B188" s="98" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C188" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D188" s="98" t="inlineStr">
+        <is>
+          <t>Api orquestadora del Gestor de Coordinación: punto único de entrada por tipo de solicitud, con el mismo rol de orquestador que los otros dos gestores.</t>
+        </is>
+      </c>
+      <c r="E188" s="126" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F188" s="98">
+        <f>IF($E188="",0,INDEX($M$5:$M$8,MATCH($E188,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G188" s="98">
+        <f>IF($F188=0,0,$F188/10)</f>
+        <v/>
+      </c>
+      <c r="H188" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C188,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I188" s="98" t="n"/>
+      <c r="J188" s="98" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K188" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="30" customHeight="1">
+      <c r="A189" s="98" t="inlineStr">
+        <is>
+          <t>RF-136</t>
+        </is>
+      </c>
+      <c r="B189" s="98" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C189" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D189" s="98" t="inlineStr">
+        <is>
+          <t>Traza de la decisión de asignación: prestador elegido, criterio aplicado, candidatos descartados y peso de cada criterio en el momento de decidir.</t>
+        </is>
+      </c>
+      <c r="E189" s="126" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F189" s="98">
+        <f>IF($E189="",0,INDEX($M$5:$M$8,MATCH($E189,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G189" s="98">
+        <f>IF($F189=0,0,$F189/10)</f>
+        <v/>
+      </c>
+      <c r="H189" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C189,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I189" s="98" t="n"/>
+      <c r="J189" s="98" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
+      <c r="K189" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="30" customHeight="1">
+      <c r="A190" s="98" t="inlineStr">
+        <is>
+          <t>RF-137</t>
+        </is>
+      </c>
+      <c r="B190" s="98" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C190" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D190" s="98" t="inlineStr">
+        <is>
+          <t>Publica al bus el evento de prestador asignado, con la llave de correlación del caso y del siniestro padre, para que la torre lo lea.</t>
+        </is>
+      </c>
+      <c r="E190" s="126" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F190" s="98">
+        <f>IF($E190="",0,INDEX($M$5:$M$8,MATCH($E190,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G190" s="98">
+        <f>IF($F190=0,0,$F190/10)</f>
+        <v/>
+      </c>
+      <c r="H190" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C190,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I190" s="98" t="n"/>
+      <c r="J190" s="98" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K190" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="30" customHeight="1">
+      <c r="A191" s="98" t="inlineStr">
+        <is>
+          <t>RF-138</t>
+        </is>
+      </c>
+      <c r="B191" s="98" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C191" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D191" s="98" t="inlineStr">
+        <is>
+          <t>Notifica al cliente el prestador asignado y cualquier cambio posterior de prestador.</t>
+        </is>
+      </c>
+      <c r="E191" s="126" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F191" s="98">
+        <f>IF($E191="",0,INDEX($M$5:$M$8,MATCH($E191,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G191" s="98">
+        <f>IF($F191=0,0,$F191/10)</f>
+        <v/>
+      </c>
+      <c r="H191" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C191,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I191" s="98" t="n"/>
+      <c r="J191" s="98" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K191" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="30" customHeight="1">
+      <c r="A192" s="98" t="inlineStr">
+        <is>
+          <t>RF-139</t>
+        </is>
+      </c>
+      <c r="B192" s="98" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="C192" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D192" s="98" t="inlineStr">
+        <is>
+          <t>Registra el cambio de prestador con su motivo, de modo que el caso conserve el histórico de asignaciones y no solo la última.</t>
+        </is>
+      </c>
+      <c r="E192" s="126" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F192" s="98">
+        <f>IF($E192="",0,INDEX($M$5:$M$8,MATCH($E192,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G192" s="98">
+        <f>IF($F192=0,0,$F192/10)</f>
+        <v/>
+      </c>
+      <c r="H192" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C192,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I192" s="98" t="n"/>
+      <c r="J192" s="98" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K192" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="30" customHeight="1">
+      <c r="A193" s="98" t="inlineStr">
+        <is>
+          <t>RT-055</t>
+        </is>
+      </c>
+      <c r="B193" s="98" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C193" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D193" s="98" t="inlineStr">
+        <is>
+          <t>Reglas de asignación versionadas con vigencia y autor, almacenadas fuera del código y expuestas como herramienta, no embebidas en lógica de aplicación.</t>
+        </is>
+      </c>
+      <c r="E193" s="126" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F193" s="98">
+        <f>IF($E193="",0,INDEX($M$5:$M$8,MATCH($E193,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G193" s="98">
+        <f>IF($F193=0,0,$F193/10)</f>
+        <v/>
+      </c>
+      <c r="H193" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C193,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I193" s="98" t="n"/>
+      <c r="J193" s="98" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
+      <c r="K193" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="30" customHeight="1">
+      <c r="A194" s="98" t="inlineStr">
+        <is>
+          <t>RT-056</t>
+        </is>
+      </c>
+      <c r="B194" s="98" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C194" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D194" s="98" t="inlineStr">
+        <is>
+          <t>Pesos del ranking como configuración y no como código, administrados por la API de gestión y configuraciones del plano de control.</t>
+        </is>
+      </c>
+      <c r="E194" s="126" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F194" s="98">
+        <f>IF($E194="",0,INDEX($M$5:$M$8,MATCH($E194,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G194" s="98">
+        <f>IF($F194=0,0,$F194/10)</f>
+        <v/>
+      </c>
+      <c r="H194" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C194,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I194" s="98" t="n"/>
+      <c r="J194" s="98" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
+      <c r="K194" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="30" customHeight="1">
+      <c r="A195" s="98" t="inlineStr">
+        <is>
+          <t>RT-057</t>
+        </is>
+      </c>
+      <c r="B195" s="98" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C195" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D195" s="98" t="inlineStr">
+        <is>
+          <t>Lectura del catálogo de red, del convenio vigente y de la tarifa por Domain API de SuraHis sobre Apigee, expuesta como herramienta en APIM.</t>
+        </is>
+      </c>
+      <c r="E195" s="126" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F195" s="98">
+        <f>IF($E195="",0,INDEX($M$5:$M$8,MATCH($E195,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G195" s="98">
+        <f>IF($F195=0,0,$F195/10)</f>
+        <v/>
+      </c>
+      <c r="H195" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C195,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I195" s="98" t="n"/>
+      <c r="J195" s="98" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K195" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="30" customHeight="1">
+      <c r="A196" s="98" t="inlineStr">
+        <is>
+          <t>RT-058</t>
+        </is>
+      </c>
+      <c r="B196" s="98" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C196" s="98" t="inlineStr">
+        <is>
+          <t>Gestor de Coordinación</t>
+        </is>
+      </c>
+      <c r="D196" s="98" t="inlineStr">
+        <is>
+          <t>Namespace propio del gestor en AKS, con imagen en Azure Container Registry, identidad técnica y secretos en Key Vault.</t>
+        </is>
+      </c>
+      <c r="E196" s="126" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F196" s="98">
+        <f>IF($E196="",0,INDEX($M$5:$M$8,MATCH($E196,$L$5:$L$8,0)))</f>
+        <v/>
+      </c>
+      <c r="G196" s="98">
+        <f>IF($F196=0,0,$F196/10)</f>
+        <v/>
+      </c>
+      <c r="H196" s="98">
+        <f>IFERROR(INDEX($O$15:$O$29,MATCH($C196,$L$15:$L$29,0)),"🟨 validar")</f>
+        <v/>
+      </c>
+      <c r="I196" s="98" t="n"/>
+      <c r="J196" s="98" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="K196" s="127" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q187"/>
+  <autoFilter ref="A4:Q196"/>
   <mergeCells count="16">
     <mergeCell ref="M48:Q48"/>
     <mergeCell ref="M40:Q40"/>
@@ -9591,12 +10651,15 @@
     <mergeCell ref="M36:Q36"/>
     <mergeCell ref="L3:N3"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="E5:E187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="E5:E196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>$L$5:$L$8</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J5:J196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Agéntica,Habilitadora,Determinística"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K5:K196" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"v1,v2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>